<commit_message>
fix(db): 한 런에서 한 TC 의 결과 행은 하나 (v1.3.1.0, SYM-5)
test_results 에 (test_run_id, test_case_id) 유니크 제약이 없었다. 결과 행을
만드는 경로가 셋인데(런 생성, 런 동기화, 결과 제출) 셋 다 조회 후 삽입이라
동시 요청에서 같은 쌍이 두 번 들어갔다. 운영 DB 에 실제로 하나 있었다
(run=25, case=5345). 중복이 있으면 리포트 total 이 부풀려지고 나머지 행은
고아 NS 로 남아 진행률을 왜곡한다.

- 마이그레이션 a1c4e7b9d2f0: 병합 후 유니크 인덱스 생성
- 병합은 삭제가 아니다. 두 행이 서로 다른 측정값을 갖고 있었다. 텍스트를
  잇고 실행 메타데이터는 실제 결과가 있는 행 것을 따르며 첨부를 옮긴다.
  결과가 서로 다르면 그 사실을 비고에 남긴다
- 런 동기화는 방언에 맞는 on_conflict_do_nothing 으로 넣는다
- 런 복제는 원본에 중복이 있어도 TC 기준 한 번만 복사한다
- 결과 제출은 유니크 위반에 한해 409 를 낸다. 다른 무결성 오류는 삼키지 않는다

운영 DB 4,338 -> 4,337행, 병합 행에 두 측정값이 모두 남았다.
테스트 224건 통과(이전 210). 신규 14건은 마이그레이션 병합 규칙과 실제
SQLite 동작까지 본다. 변이 7종으로 이빨을 확인했다.
회귀 체크리스트에 TC-RUN-021 추가. QA 2인 통과.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYLhfQkmoR154wEzgockv5
</commit_message>
<xml_diff>
--- a/TC_Manager_Full_Regression_Checklist.xlsx
+++ b/TC_Manager_Full_Regression_Checklist.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="체크리스트" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인코딩이슈추적" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="체크리스트" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="인코딩이슈추적" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="요약" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'체크리스트'!$A$2:$O$2</definedName>
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O174"/>
+  <dimension ref="A1:O175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10292,6 +10292,68 @@
       <c r="M174" s="6" t="n"/>
       <c r="N174" s="6" t="n"/>
       <c r="O174" s="6" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="B175" s="6" t="inlineStr">
+        <is>
+          <t>TC-RUN-021</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="inlineStr">
+        <is>
+          <t>테스트 런</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t>결과 무결성</t>
+        </is>
+      </c>
+      <c r="E175" s="6" t="inlineStr">
+        <is>
+          <t>한 런에서 한 TC 의 결과 행은 하나만 생긴다</t>
+        </is>
+      </c>
+      <c r="G175" s="6" t="inlineStr">
+        <is>
+          <t>기능</t>
+        </is>
+      </c>
+      <c r="H175" s="7" t="inlineStr">
+        <is>
+          <t>진행 중인 런과 그 프로젝트에 TC 가 하나 이상 있음</t>
+        </is>
+      </c>
+      <c r="I175" s="7" t="inlineStr">
+        <is>
+          <t>1. 런 상세를 두 브라우저 탭에서 거의 동시에 연다(런 동기화가 각각 호출된다).
+2. 같은 TC 의 결과를 두 탭에서 거의 동시에 저장한다.
+3. 런을 복제한다.
+4. DB 에서 test_results 를 (test_run_id, test_case_id) 로 묶어 센다.</t>
+        </is>
+      </c>
+      <c r="J175" s="7" t="inlineStr">
+        <is>
+          <t>1. 어느 경로에서도 같은 (런, TC) 결과 행이 둘 이상 생기지 않는다.
+2. 동시 저장이 겹치면 500 이 아니라 409 와 재시도 안내가 나온다.
+3. 리포트의 total 이 실제 TC 수와 일치한다.</t>
+        </is>
+      </c>
+      <c r="L175" s="8" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="O175" s="6" t="inlineStr">
         <is>
           <t>높음</t>
         </is>

</xml_diff>